<commit_message>
Update Ibis Jaipur price history
</commit_message>
<xml_diff>
--- a/Accor_Ibis_Jaipur_Price_History.xlsx
+++ b/Accor_Ibis_Jaipur_Price_History.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K297"/>
+  <dimension ref="A1:K298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14977,6 +14977,55 @@
         </is>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:11:51</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>4</v>
+      </c>
+      <c r="E298" t="n">
+        <v>2</v>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>2,2</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>ibis Jaipur City Centre</t>
+        </is>
+      </c>
+      <c r="H298" t="n">
+        <v>5506</v>
+      </c>
+      <c r="I298" t="n">
+        <v>5795</v>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Official Accor displayed stay price</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>